<commit_message>
Read/Write for main program
Finished implementation of read/write for main program.
Sorted out some of the data.
Fixed bug in student class
</commit_message>
<xml_diff>
--- a/test_data/preferences_data.xlsx
+++ b/test_data/preferences_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tom\Documents\GitHub\GRG23VBS-Berufsorientierungstage-Zuteilung\test_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59E155FC-1330-4109-902E-A9007F592682}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{605764B9-C8D8-41D0-B7FD-7D433BB6A43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-3398" yWindow="8002" windowWidth="20716" windowHeight="13155" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,45 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="27">
   <si>
-    <t>FirstName</t>
-  </si>
-  <si>
-    <t>LastName</t>
-  </si>
-  <si>
-    <t>Year</t>
-  </si>
-  <si>
-    <t>Wish 1</t>
-  </si>
-  <si>
-    <t>Wish 2</t>
-  </si>
-  <si>
-    <t>Wish 3</t>
-  </si>
-  <si>
-    <t>Wish 4</t>
-  </si>
-  <si>
-    <t>Wish 5</t>
-  </si>
-  <si>
-    <t>Wish 6</t>
-  </si>
-  <si>
-    <t>Wish 7</t>
-  </si>
-  <si>
-    <t>Wish 8</t>
-  </si>
-  <si>
-    <t>Wish 9</t>
-  </si>
-  <si>
-    <t>Wish 10</t>
-  </si>
-  <si>
     <t>F1</t>
   </si>
   <si>
@@ -106,6 +67,45 @@
   </si>
   <si>
     <t>Workshop2</t>
+  </si>
+  <si>
+    <t>Vorname</t>
+  </si>
+  <si>
+    <t>Nachname</t>
+  </si>
+  <si>
+    <t>Klasse</t>
+  </si>
+  <si>
+    <t>Wunsch 1</t>
+  </si>
+  <si>
+    <t>Wunsch 2</t>
+  </si>
+  <si>
+    <t>Wunsch 3</t>
+  </si>
+  <si>
+    <t>Wunsch 4</t>
+  </si>
+  <si>
+    <t>Wunsch 5</t>
+  </si>
+  <si>
+    <t>Wunsch 6</t>
+  </si>
+  <si>
+    <t>Wunsch 7</t>
+  </si>
+  <si>
+    <t>Wunsch 8</t>
+  </si>
+  <si>
+    <t>Wunsch 9</t>
+  </si>
+  <si>
+    <t>Wunsch 10</t>
   </si>
 </sst>
 </file>
@@ -439,125 +439,125 @@
   <sheetData>
     <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>21</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>22</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="K1" t="s">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="M1" t="s">
-        <v>12</v>
+        <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>7</v>
       </c>
       <c r="D2" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="E2" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="G2" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="H2" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="I2" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="J2" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="K2" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="L2" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="M2" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="C3">
         <v>7</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
+        <v>4</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="G3" t="s">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="H3" t="s">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="I3" t="s">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="J3" t="s">
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="K3" t="s">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c r="L3" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="M3" t="s">
-        <v>19</v>
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>